<commit_message>
feat: interactive SKU substitution table, instant dialog, CSR scroll-to-top, pipeline enhancements
- Replace static obsolete-SKU table + separate radio list with a single interactive bordered table (radio-select column, pricing, View details popup per row); remove Compatibility column and AI pick badge
- View details dialog opens instantly (CSS animation/transition disabled)
- Auto-scroll to CSR DECISION NEEDED banner for all intake and pipeline exception cards
- Fix double line separator after Source/Extraction method caption
- Remove PN-DRAIN-STD SKU not found scenario from demo PO (use valid SKU-DRN-3010)
- Stock availability hard-stop during product matching; split-shipment CSR gate; budget/approval-matrix moved to last pipeline stage
- Updated master data, inventory splits, and intake resolver ordering

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/mock-data/compliance-master-data.xlsx
+++ b/mock-data/compliance-master-data.xlsx
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1120,7 +1120,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>SKU-DRN-3010</t>
+          <t>SKU-CTG-1017</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SKU-VLV-2201</t>
+          <t>SKU-DRN-3010</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>SKU-SHS-7700</t>
+          <t>SKU-DRN-7213</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>SKU-SEL-1150</t>
+          <t>SKU-VLV-2201</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1208,12 +1208,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>SKU-FIN-9100</t>
+          <t>SKU-SHS-7700</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1223,29 +1223,29 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>SDS must be attached</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>SKU-FIN-9100</t>
+          <t>SKU-SEL-1150</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Restricted - requires compliance approval</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -1257,15 +1257,59 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>SDS must be attached</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9100</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Restricted - requires compliance approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9100</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Export prohibited without licence</t>
         </is>

</xml_diff>